<commit_message>
updated the logo and title
</commit_message>
<xml_diff>
--- a/client/public/samples/bulk-offers-sample.xlsx
+++ b/client/public/samples/bulk-offers-sample.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Offers" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <si>
     <t>fullName</t>
   </si>
@@ -34,16 +34,16 @@
     <t>templateName</t>
   </si>
   <si>
-    <t>Vikram Singh</t>
-  </si>
-  <si>
-    <t>vikram.singh@example.com</t>
-  </si>
-  <si>
-    <t>UI/UX Designer</t>
-  </si>
-  <si>
-    <t>Design</t>
+    <t>Asha Reddy</t>
+  </si>
+  <si>
+    <t>asha.reddy@example.com</t>
+  </si>
+  <si>
+    <t>Medical Representative</t>
+  </si>
+  <si>
+    <t>Sales</t>
   </si>
   <si>
     <t>2026-08-01</t>
@@ -52,37 +52,34 @@
     <t>Engineering-V2</t>
   </si>
   <si>
-    <t>Rajesh Kumar</t>
-  </si>
-  <si>
-    <t>rajesh.k@example.com</t>
-  </si>
-  <si>
-    <t>DevOps Specialist</t>
-  </si>
-  <si>
-    <t>Engineering</t>
-  </si>
-  <si>
-    <t>2026-08-15</t>
-  </si>
-  <si>
-    <t>Asha Rao</t>
-  </si>
-  <si>
-    <t>asha.rao@example.com</t>
-  </si>
-  <si>
-    <t>Account Executive</t>
-  </si>
-  <si>
-    <t>Sales</t>
-  </si>
-  <si>
-    <t>2026-09-01</t>
-  </si>
-  <si>
-    <t>Sales-Standard</t>
+    <t>Rahul Mehta</t>
+  </si>
+  <si>
+    <t>rahul.mehta@example.com</t>
+  </si>
+  <si>
+    <t>HR Executive</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
+    <t>2026-09-15</t>
+  </si>
+  <si>
+    <t>Priya Nair</t>
+  </si>
+  <si>
+    <t>priya.nair@example.com</t>
+  </si>
+  <si>
+    <t>Quality Analyst</t>
+  </si>
+  <si>
+    <t>Operations</t>
+  </si>
+  <si>
+    <t>2026-10-01</t>
   </si>
 </sst>
 </file>
@@ -466,7 +463,13 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="7" width="18" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -506,7 +509,7 @@
         <v>10</v>
       </c>
       <c r="E2">
-        <v>1000000</v>
+        <v>600000</v>
       </c>
       <c r="F2" t="s">
         <v>11</v>
@@ -529,7 +532,7 @@
         <v>16</v>
       </c>
       <c r="E3">
-        <v>1400000</v>
+        <v>750000</v>
       </c>
       <c r="F3" t="s">
         <v>17</v>
@@ -552,13 +555,13 @@
         <v>21</v>
       </c>
       <c r="E4">
-        <v>800000</v>
+        <v>900000</v>
       </c>
       <c r="F4" t="s">
         <v>22</v>
       </c>
       <c r="G4" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>